<commit_message>
HVAC ideation: batch 1 briefs fact-checked, 47 fixes (safety, prices, sources)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011ZVfQJsvpiS3xEpn6GjD8a
</commit_message>
<xml_diff>
--- a/studies/hvac/ideation/batch1-briefs-2026-10-26.xlsx
+++ b/studies/hvac/ideation/batch1-briefs-2026-10-26.xlsx
@@ -458,7 +458,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Nine everyday thermostat habits that make a furnace run harder, cycle more or overheat, each with what it costs and the better setting. 1) Cranking it to 80 to warm up faster: a furnace delivers heat at one rate, so it only runs longer and overshoots; set the temperature you want. 2) Fan set to ON instead of AUTO all winter: the blower runs 24 hours a day, so older single-speed motors wear out sooner (a blower motor runs about $400-$900 installed) and the bill rises; use AUTO unless the blower is variable-speed. 3) A thermostat on an outside wall, near a lamp, a TV, a sunny window or a supply vent: false readings cause short cycling; move it or shield it. 4) Constant up-and-down adjusting through the day: every start is the hardest moment for the igniter and blower; pick a schedule and leave it. 5) Short cycling from a cycle-rate or swing setting that's too tight on digital thermostats: check the installer menu (cycles per hour) against the furnace manual. 6) Closing the vents and doors of unused rooms to 'save' heat: raises static pressure, the heat exchanger runs hot and the high limit trips; keep at least 80-90% of supply vents open. 7) Letting thermostat batteries die: the heat can drop out on the coldest night; replace them every fall ($5). 8) A smart thermostat with no C-wire 'stealing' power: can make some furnaces chatter or short cycle; add a C-wire or adapter ($20-$30). 9) Shutting the heat off completely when away in deep cold: a long, hard recovery and a frozen-pipe risk; set back 7-10°F instead (the DOE says a 7-10°F setback for 8 hours a day saves up to about 10% a year). Habits, not repairs; no item numbers in the title.</t>
+          <t>Nine everyday thermostat habits that make a furnace run harder, cycle more or overheat, each with what it costs and the better setting. 1) Cranking it to 80 to warm up faster: a single-stage furnace delivers heat at one rate (two-stage and modulating ones don't reach the set point faster either), so it only runs longer and overshoots; set the temperature you want. 2) Fan set to ON instead of AUTO all winter: the blower runs 24 hours a day, so older single-speed motors wear out sooner (a blower motor runs about $300-$1,100 installed for a standard motor, $600-$1,500+ for a variable-speed ECM) and the bill rises; use AUTO unless the blower is variable-speed. 3) A thermostat on an outside wall, near a lamp, a TV, a sunny window or a supply vent: false readings cause short cycling; move it or shield it. 4) Constant up-and-down adjusting through the day: every start is the hardest moment for the igniter and blower; pick a schedule and leave it. 5) Short cycling from a cycle-rate or swing setting that's too tight on digital thermostats: check the installer menu (cycles per hour) against the furnace manual. 6) Closing the vents and doors of unused rooms to 'save' heat: raises static pressure, the heat exchanger runs hot and the high limit trips; keep at least 80-90% of supply vents open. 7) Letting thermostat batteries die: the heat can drop out on the coldest night; replace them every fall ($5). 8) A smart thermostat with no C-wire 'stealing' power: can make some furnaces chatter or short cycle; add a C-wire or adapter ($20-$30). 9) Shutting the heat off completely when away in deep cold: the real risk is frozen pipes and a cold house if the furnace won't restart; a 7-10°F setback is the safe way to save (the DOE says a 7-10°F setback for 8 hours a day saves as much as 10% a year, and that a furnace 'working harder to recover' is a misconception). Habits, not repairs; no item numbers in the title.</t>
         </is>
       </c>
     </row>
@@ -475,7 +475,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Nine checks before the first hard cold, each with what it costs if skipped and the fix. 1) Put in a fresh filter: a clogged filter is the most common cause of a furnace overheating and shutting off on its high limit; $5-$15 against a $100-$200 service call. 2) Test-run the heat on a mild day: find a dead igniter or flame sensor now, not at 2 a.m. when emergency rates run $200-$400 just to show up. 3) Clear the intake and exhaust pipes outside (high-efficiency furnaces with white PVC pipes): leaves, nests or snow make the furnace shut itself off; keep 12 inches clear of snow. 4) Flush the condensate drain and trap with vinegar (condensing furnaces only): a clogged trap stops the furnace and can leak. 5) Test every carbon monoxide detector and replace batteries; one on every sleeping floor. 6) Open and clear every supply vent and return grille; furniture and rugs off them. 7) Replace thermostat batteries. 8) Clear 3 feet around the furnace: no paint, gas cans, laundry piles or cardboard against it. 9) Know where the furnace's power switch (looks like a light switch, often by the furnace or at the stairs) and the gas shutoff are: a switched-off furnace or tripped breaker is a common no-heat call that costs a full visit. Optional tenth for the script: book the yearly inspection before the rush, about $80-$200, which checks the heat exchanger and burners. Safety: if you smell gas, leave the house and call the gas company from outside.</t>
+          <t>Nine checks before the first hard cold, each with what it costs if skipped and the fix. 1) Put in a fresh filter: a clogged filter is the most common cause of a furnace overheating and shutting off on its high limit; $5-$15 against a $75-$200 service call. 2) Test-run the heat on a mild day: find a dead igniter or flame sensor now, not at 2 a.m. when an emergency visit runs $250-$400 or more. 3) Clear the intake and exhaust pipes outside (high-efficiency furnaces with white PVC pipes): leaves, nests or snow make the furnace shut itself off; keep the pipe ends at least 12 inches above the snow line and clear. 4) Flush the condensate drain and trap with vinegar (condensing furnaces only), then refill the trap with water so it's primed: a clogged trap stops the furnace and can leak, and an empty trap can stop it too or let exhaust escape. 5) Test every carbon monoxide alarm: one on every level of the home and outside each sleeping area (CPSC); replace batteries, or the whole alarm if it's past its end-of-life date (most last 5-10 years). 6) Open and clear every supply vent and return grille; furniture and rugs off them. 7) Replace thermostat batteries. 8) Clear 3 feet around the furnace: no paint, gas cans, laundry piles or cardboard against it. 9) Know where the furnace's power switch (looks like a light switch, often by the furnace or at the stairs) and the gas shutoff are: a switched-off furnace or tripped breaker is a common no-heat call that costs a full visit. Optional tenth for the script: book the yearly inspection before the rush, about $80-$250, which checks the heat exchanger and burners. Safety: if you smell gas, leave the house and call the gas company from outside.</t>
         </is>
       </c>
     </row>
@@ -492,7 +492,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>The filter's main job is protecting the blower and heat exchanger, and a plain pleated MERV 8 filter (about $5-$8 each in a multipack) does that while letting air through. Many 1-inch 'allergen' or 'MERV 13' filters at $20-$35 each are dense enough to restrict airflow on the average home system, whose ducts and blower were sized for a low-resistance filter: higher static pressure, the blower straining, the heat exchanger running hot and tripping the high limit, and in summer a frozen AC coil. The worst case is a premium filter left in too long. The cheapest fiberglass filters ($1-$3) are the other extreme: they stop big debris but let fine dust coat the blower wheel and coil. How to choose: check the furnace manual for the recommended MERV; MERV 8 for most homes; change 1-inch filters every 1-3 months (monthly with pets); if you want cleaner air for allergies, a 4-5 inch media cabinet (filters about $25-$60, last 6-12 months) or a standalone HEPA room purifier ($100-$250) does it without choking the furnace. Honest limits: a high-MERV filter is fine on a system built for it; the point is matching the filter to the system. A blower motor replacement runs about $400-$900; a heat exchanger failure often means a new furnace.</t>
+          <t>The filter's main job is protecting the blower and heat exchanger, and a plain pleated MERV 8 filter (about $5-$8 each in a multipack) does that while letting air through. A dense 1-inch 'allergen' or MERV 11-13 filter at $20-$35 adds resistance: in studies it cut airflow by roughly 7-11% on common single-speed (PSC) blowers, and on systems with small or few return grilles that can push the furnace toward overheating and high-limit trips, and in summer a frozen AC coil. The EPA recommends MERV 13 or as high as the system fan and filter slot can handle, so check the furnace manual or ask a tech. The worst case is a premium filter left in too long. The cheapest fiberglass filters ($1-$3) are the other extreme: they stop big debris but let fine dust coat the blower wheel and coil. How to choose: check the furnace manual for the recommended MERV; MERV 8 for most homes; change 1-inch filters every 1-3 months (monthly with pets); if you want cleaner air for allergies, a 4-5 inch media cabinet (filters about $25-$60, last 6-12 months) or a standalone HEPA room purifier ($100-$250) does it without choking the furnace. Honest limits: a high-MERV filter is fine on a system built for it; the point is matching the filter to the system. A blower motor replacement runs about $300-$1,100 (variable-speed ECM $600-$1,500+); a heat exchanger failure often means a new furnace.</t>
         </is>
       </c>
     </row>
@@ -509,7 +509,7 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Eleven homeowner mistakes that lead to service calls, each with the cost and the fix. 1) Running a dirty filter: overheating and limit trips; $5-$15 filter vs a $100-$200 call. 2) Closing vents in unused rooms: high static pressure, overheating. 3) Blocking return grilles with furniture. 4) Never looking at the condensate trap on a high-efficiency furnace: a clog shuts it down; a vinegar flush costs pennies. 5) Letting snow, leaves or nests block the PVC intake and exhaust pipes. 6) Calling for 'no heat' when the furnace switch was turned off or the breaker tripped: check both first. 7) Paying $150-$300 to replace a flame sensor that only needed cleaning (a $10-$25 part, cleaned with fine emery cloth or steel wool). 8) Accepting a replacement quote for an igniter failure: a hot-surface igniter is a $20-$60 part, about $150-$350 installed. 9) Agreeing to a new furnace on a verbal 'cracked heat exchanger' without photos, a camera inspection or a second opinion (a cracked heat exchanger is a real CO danger; insist on seeing the proof). 10) Thermostat fan left ON all season. 11) Storing boxes, paint and laundry against the furnace. The adversary is the business model that profits from avoidable calls, not every technician; recommend a yearly inspection by someone you trust. Prices as rounded ranges.</t>
+          <t>Eleven homeowner mistakes that lead to service calls, each with the cost and the fix. 1) Running a dirty filter: overheating and limit trips; $5-$15 filter vs a $75-$200 call. 2) Closing vents in unused rooms: high static pressure, overheating. 3) Blocking return grilles with furniture. 4) Never looking at the condensate trap on a high-efficiency furnace: a clog shuts it down; a vinegar flush costs pennies (refill the trap with water afterwards). 5) Letting snow, leaves or nests block the PVC intake and exhaust pipes. 6) Calling for 'no heat' when the furnace switch was turned off or the breaker tripped: check both first. 7) Paying $100-$250 for a flame sensor job when it often only needs cleaning (a $10-$25 part, cleaned with a Scotch-Brite pad or very fine emery cloth). 8) Accepting a replacement quote for an igniter failure: a hot-surface igniter is a $20-$60 part, about $120-$350 installed. 9) Agreeing to a new furnace on a verbal 'cracked heat exchanger' without photos, a camera inspection or a second opinion (a cracked heat exchanger is a real CO danger; insist on seeing the proof, but if a tech red-tags the furnace or your CO alarm goes off, don't run it while you wait for the second opinion). 10) Thermostat fan left ON all season. 11) Storing boxes, paint and laundry against the furnace. The adversary is the business model that profits from avoidable calls, not every technician; recommend a yearly inspection by someone you trust. Prices as rounded ranges.</t>
         </is>
       </c>
     </row>
@@ -526,7 +526,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>The substance is plain white vinegar. Only high-efficiency condensing furnaces (90%+ AFUE, white PVC vent pipes) make water: a few gallons a day in cold weather, drained through a plastic trap, a hose and often a small condensate pump. Over a season, slime and biofilm grow in the trap and line. When it clogs, the water backs up, the pressure switch can't close and the furnace shuts down or flashes an error code, or the trap overflows onto the floor. A clogged-condensate service call runs about $150-$300; a failed condensate pump $100-$250 installed; water damage under a basement furnace much more. The fix: turn the furnace off, find the cleanout or vent tee on the drain line or remove the trap per the manual, pour about a cup of white vinegar in, wait 30 minutes, then flush with a cup or two of warm water; once a month or two in the heating season. Why not bleach: many manufacturers recommend vinegar or plain water, bleach fumes in a closed utility room and its effect on some metal and rubber parts are the reasons usually given; never mix bleach and vinegar (toxic chlorine gas). Note: standard 80% furnaces have no condensate drain of their own (the AC coil drain above them is a separate summer job).</t>
+          <t>The substance is plain white vinegar. Only high-efficiency condensing furnaces (90%+ AFUE, white PVC vent pipes) make water: a few gallons a day in cold weather, drained through a plastic trap, a hose and often a small condensate pump. Over a season, slime and biofilm grow in the trap and line. When it clogs, the water backs up, the pressure switch can't close and the furnace shuts down or flashes an error code, or the trap overflows onto the floor. A clogged-condensate service call runs about $150-$300; a failed condensate pump about $150-$400 installed; water damage under a basement furnace much more. The fix: turn the furnace off, find the cleanout or vent tee on the drain line or remove the trap per the manual, pour about a cup of white vinegar in, wait 30 minutes, then flush with a cup or two of warm water; once a month or two in the heating season. Why not bleach: Carrier and Lennox recommend white vinegar over bleach for condensate lines (Carrier: harsh chemicals can damage system components), and furnace manuals usually call for plain water in the trap; never mix bleach and vinegar (toxic chlorine gas). Make sure the trap is full of water before restoring power, and pour only into the drain cleanout or vent tee, never into the rubber pressure-switch hoses or the inducer. The title's 'all winter' is delivered as a cup once a month through the heating season; the script says so plainly. Note: standard 80% furnaces have no condensate drain of their own (the AC coil drain above them is a separate summer job).</t>
         </is>
       </c>
     </row>
@@ -543,7 +543,7 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>What comes out of a high-efficiency furnace's condensate drain after a vinegar flush: the slime, algae-like biofilm and sludge that grow in the trap and line, sometimes rust flakes from a metal drain pan, and occasionally an insect nest at the outdoor end. It matters because the furnace makes a few gallons of slightly acidic water a day in cold weather; a clogged trap makes the pressure switch open and the furnace shut down, short cycle or show an error code, and it can overflow. How: turn the furnace off; locate the trap and the drain line (where it ends: a floor drain, condensate pump or outside); pour about a cup of white vinegar into the cleanout or vent tee, wait 30 minutes, flush with warm water and watch the outlet. If it barely drains, the trap may need removing and rinsing per the manual, or a wet-dry vacuum on the outside end of the line. Costs: a clogged-condensate call about $150-$300, a condensate pump about $100-$250 installed. Only condensing furnaces (90%+ AFUE, PVC vent pipes) have this drain. Safety: never mix vinegar with bleach; power off before opening the trap.</t>
+          <t>What comes out of a high-efficiency furnace's condensate drain after a vinegar flush: the slime, algae-like biofilm and sludge that grow in the trap and line, sometimes debris from the AC coil's pan above it, and occasionally an insect nest at the outdoor end. It matters because the furnace makes a few gallons of slightly acidic water a day in cold weather; a clogged trap makes the pressure switch open and the furnace shut down, short cycle or show an error code, and it can overflow. How: turn the furnace off; locate the trap and the drain line (where it ends: a floor drain, condensate pump or outside); pour about a cup of white vinegar into the cleanout or vent tee, wait 30 minutes, flush with warm water and watch the outlet; refill the trap with water before restoring power, and never pour into the rubber pressure-switch hoses or the inducer. If it barely drains, the trap may need removing and rinsing per the manual, or a wet-dry vacuum on the outside end of the line. Costs: a clogged-condensate call about $150-$300, a condensate pump about $150-$400 installed. Only condensing furnaces (90%+ AFUE, PVC vent pipes) have this drain. Safety: never mix vinegar with bleach; power off before opening the trap.</t>
         </is>
       </c>
     </row>
@@ -560,7 +560,7 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Eleven honest HVAC uses for a few drops of dish soap in water. 1) Leak-check the gas fittings after any work: brush soapy water on the joints; growing bubbles mean a leak (if you smell gas, leave and call the gas company; never use a flame). 2) Leak-check the refrigerant line connections the same way; techs use bubble solution for this. 3) Wash a reusable (washable) furnace or mini-split filter, then dry it completely before refitting. 4) Clean the outdoor unit's coil gently: mild soapy water, low-pressure garden hose, rinse from inside out, power off at the disconnect (a pro coil cleaning runs $100-$200+). 5) Clean return grilles and supply registers (grease and dust film). 6) Clean the AC condensate drain pan before the vinegar flush. 7) Clean window-AC and dehumidifier filters. 8) Wipe down the furnace cabinet and blower door so dust doesn't get drawn in. 9) Clean the dehumidifier bucket and humidifier water tray (rinse well). 10) Clean the condensate pump's reservoir: unplug it, rinse the tank with warm soapy water, rinse clear, refit (a clogged pump stops the furnace or AC and overflows). 11) Clean ceiling-fan blades before reversing them for winter. Honest framing: soap is a cleaner and a leak finder, never a fix for a gas or refrigerant leak; those need a licensed pro. No dish soap inside the furnace's burner compartment.</t>
+          <t>Eleven honest HVAC uses for a few drops of dish soap in water. 1) Spot-check visible gas fittings with very mild soapy water or, better, a non-corrosive leak-check solution from the hardware store (some soaps can corrode brass and CSST fittings), then wipe it off; growing bubbles mean a leak (if you smell gas, leave and call the gas company; never use a flame; any gas work itself is for a licensed pro). 2) Leak-check the refrigerant line connections the same way; techs use bubble solution for this. 3) Wash a reusable (washable) furnace or mini-split filter, then dry it completely before refitting. 4) Clean the outdoor unit's coil gently: mild soapy water, low-pressure garden hose, rinse from inside out only if the top lifts off without straining the fan wires, otherwise spray gently from outside in; power off at the disconnect (a pro coil cleaning runs $100-$200+). 5) Clean return grilles and supply registers (grease and dust film). 6) Clean the AC condensate drain pan before the vinegar flush. 7) Clean window-AC and dehumidifier filters. 8) Wipe down the furnace cabinet and blower door so dust doesn't get drawn in. 9) Clean the dehumidifier bucket and humidifier water tray (rinse well). 10) Clean the condensate pump's reservoir: unplug it, rinse the tank with warm soapy water, rinse clear, refit (a clogged pump stops the furnace or AC and overflows). 11) Clean ceiling-fan blades before reversing them for winter. Honest framing: soap is a cleaner and a leak finder, never a fix for a gas or refrigerant leak; those need a licensed pro. No dish soap inside the furnace's burner compartment.</t>
         </is>
       </c>
     </row>
@@ -577,7 +577,7 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Roger's monthly habit in the heating season: a cup of white vinegar into his high-efficiency furnace's condensate trap and line, then warm water. The thousands it saves, item by item: no clogged-condensate service calls (about $150-$300 each, more on a weekend or night); no replaced pressure switch (about $150-$350 installed) or condensate pump (about $100-$250); no water damage under a basement furnace or in a finished room (drywall, flooring, mold remediation can run into the thousands); no frozen house from a furnace that shut itself down on the coldest night. How: power off, pour through the cleanout or vent tee, wait 30 minutes, flush, check the outlet runs freely; in summer the same habit on the AC coil's drain line. Only condensing furnaces (90%+ AFUE, white PVC vent pipes) have this drain. Never mix vinegar and bleach. Persona narrative only: it's his routine, not a filmed test.</t>
+          <t>Roger's monthly habit in the heating season: a cup of white vinegar into his own high-efficiency furnace's condensate trap and line, then warm water. The thousands it saves, item by item: no clogged-condensate service calls (about $150-$300 each, more on a weekend or night); no water drawn into the pressure-switch hose, which can ruin the switch (about $175-$350 installed), and no condensate pump (about $150-$400 installed); no water damage under a basement furnace or in a finished room (drywall, flooring and mold remediation are where the thousands are; keep that line explicit); no frozen house from a furnace that shut itself down on the coldest night. How: power off, pour through the cleanout or vent tee, wait 30 minutes, flush, refill the trap with water, check the outlet runs freely; in summer the same habit on the AC coil's drain line. Only condensing furnaces (90%+ AFUE, white PVC vent pipes) have this drain. Never mix vinegar and bleach. Persona narrative only: it's his routine, not a filmed test.</t>
         </is>
       </c>
     </row>
@@ -594,7 +594,7 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>A persona verdict, ranked worst to best for the furnace. Fiberglass (about $1-$3, MERV 1-4): lets air through easily but catches only big debris; fine dust coats the blower and coil; acceptable only if changed monthly. Washable / electrostatic ($20-$50 once): low filtration, must be washed and dried completely (a damp filter grows mold and restricts air), and charge fades; not worth it for most. 'HEPA' 1-inch filters: true HEPA is far too restrictive for a typical home furnace without a dedicated bypass or system built for it, so most 'HEPA-type' 1-inch filters are marketing; real HEPA belongs in a standalone room purifier ($100-$250). Pleated MERV 8 (about $5-$8 each in a multipack): the winner for most homes; catches dust, pollen and mold spores while keeping airflow; MERV 11-13 only if the system is rated for it or in a 4-5 inch media cabinet. Change 1-inch filters every 1-3 months. Costs of the wrong pick: overheating and limit trips, a blower motor at about $400-$900. Verdict delivered as research and experience, never a filmed test. Tenure number '45' is a placeholder until set.</t>
+          <t>A persona verdict, ranked worst to best for the furnace. Fiberglass (about $1-$3, MERV 1-4): lets air through easily but catches only big debris; fine dust coats the blower and coil; acceptable only if changed monthly. Washable / electrostatic ($20-$50 once): low filtration, must be washed and dried completely (a damp filter grows mold and restricts air), and charge fades; not worth it for most. 'HEPA' 1-inch filters: true HEPA is far too restrictive for a typical home furnace without a dedicated bypass or system built for it, so most 'HEPA-type' 1-inch filters are marketing; real HEPA belongs in a standalone room purifier ($100-$250). Pleated MERV 8 (about $5-$8 each in a multipack): the winner for most homes; catches dust, pollen and mold spores while keeping airflow; MERV 11-13 if the system is rated for it or in a 4-5 inch media cabinet (the EPA recommends MERV 13 or the highest the system can handle, so the ranking is about fit, not anti-MERV-13). Change 1-inch filters every 1-3 months. Costs of the wrong pick: overheating and limit trips, a blower motor at about $300-$1,100 (variable-speed $600-$1,500+). Verdict delivered as research and experience, never a filmed test. Tenure number '45' is a placeholder until set.</t>
         </is>
       </c>
     </row>
@@ -611,7 +611,7 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>The $5 monthly habit: a five-minute look on the first of each month in the heating season. Pull the filter and hold it to the light; replace it if light barely passes ($5-$8 for a pleated MERV 8). Glance at the condensate trap and line on a high-efficiency furnace and flush with a cup of vinegar if it's slow. Look outside at the PVC intake and exhaust pipes for snow, ice or nests. Look through the sight glass at the flame or listen to a full cycle: a steady start and no repeated restarts. Check the thermostat batteries and that the fan is on AUTO. Why it works: many common winter no-heat calls come from a clogged filter, a blocked drain or vent pipe, a dirty flame sensor or a tripped switch, all cheap to prevent; a winter no-heat call costs $100-$200 for the visit alone, $200-$400 at night or on a weekend. 'Never break down' is puffery: the honest claim is far fewer breakdowns; parts still wear out, and a yearly inspection ($80-$200) still checks the heat exchanger and burners.</t>
+          <t>The $5 monthly habit: a five-minute look on the first of each month in the heating season. Pull the filter and hold it to the light; replace it if light barely passes ($5-$8 for a pleated MERV 8). Glance at the condensate trap and line on a high-efficiency furnace and flush with a cup of vinegar if it's slow, then refill the trap with water. Look outside at the PVC intake and exhaust pipes for snow, ice or nests. Look through the sight glass at the flame or listen to a full cycle: a steady start and no repeated restarts. Check the thermostat batteries and that the fan is on AUTO. Why it works: many common winter no-heat calls come from a clogged filter, a blocked drain or vent pipe, a dirty flame sensor or a tripped switch, all cheap to prevent; a winter no-heat call costs $75-$200 for the visit alone, $250-$400 or more at night or on a weekend. 'Never break down' is puffery: the honest claim is far fewer breakdowns; parts still wear out, and a yearly inspection ($80-$250) still checks the heat exchanger and burners.</t>
         </is>
       </c>
     </row>
@@ -628,7 +628,7 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>The leak is the rim joist (band joist): the wooden band sitting on top of the foundation wall around the basement or crawlspace, often with no insulation and gaps at the sill plate, wire and pipe holes. Warm air rises and escapes at the top of the house, and this stack effect pulls cold air in low, through those gaps, so the furnace keeps reheating outside air. ENERGY STAR estimates homeowners can save an average of 15% on heating and cooling costs (about 11% of total energy costs) by air sealing and insulating attics, floors over crawlspaces and basement rim joists. The fix: canned spray foam (about $5-$10 a can) in the gaps and holes, or rigid foam board cut to fit each joist bay and sealed with foam around the edges ($20-$60 for a typical section, more for a whole house); a pro spray-foam job runs much higher. How to find it: on a cold windy day, feel along the top of the basement wall or use an incense stick. Safety: keep foam away from flue pipes, the furnace and water-heater vents (clearances), and many codes require exposed foam board to be covered with a fire-rated barrier; wear gloves and eye protection.</t>
+          <t>The leak is the rim joist (band joist): the wooden band sitting on top of the foundation wall around the basement or crawlspace, often with no insulation and gaps at the sill plate, wire and pipe holes. Warm air rises and escapes at the top of the house, and this stack effect pulls cold air in low, through those gaps, so the furnace keeps reheating outside air. ENERGY STAR estimates homeowners can save an average of 15% on heating and cooling costs (about 11% of total energy costs) by air sealing and insulating attics, floors over crawlspaces and basement rim joists; the script attributes this to the whole package, never to the rim joist alone. The fix: canned spray foam (about $5-$10 a can) in the gaps and holes, or rigid foam board cut to fit each joist bay and sealed with foam around the edges ($20-$60 for a typical section, more for a whole house); a pro spray-foam job runs much higher. How to find it: on a cold windy day, feel along the top of the basement wall or use an incense stick. Safety: if the furnace or water heater is an older natural-draft type (a metal vent into a chimney), sealing the basement tighter can make it backdraft carbon monoxide (ENERGY STAR warns of this): have a combustion safety (draft) test done and keep working CO alarms. Canned foam is flammable while curing: no flames or pilot lights nearby, ventilate. Around flues use sheet metal and high-temperature fire-rated sealant, never foam; many codes require exposed foam board to be covered with a fire-rated barrier; gloves and eye protection.</t>
         </is>
       </c>
     </row>
@@ -645,7 +645,7 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Seven cheap fixes for the drafts that make a house feel cold, set against a typical whole-house insulation quote (blown-in or spray foam often runs several thousand dollars). 1) Door weatherstripping and a door sweep ($10-$25 a door): the biggest felt draft in most homes. 2) Foam gaskets behind outlet and switch covers on outside walls ($5 for a pack). 3) Caulk the window and door trim where it meets the wall ($5-$10 a tube). 4) Window insulation film kits ($15-$25 for several windows) or heavy thermal curtains. 5) Weatherstrip and insulate the attic hatch or pull-down stairs ($20-$50): often a big hole in the ceiling. 6) Seal the basement rim joist with canned foam ($5-$10 a can). 7) Close the fireplace damper or fit a chimney plug ($30-$80) when the fire is out. Honest framing: these stop air leaks, which cause most of the 'cold house' feeling; they don't replace insulation in a truly empty wall or attic, and an energy audit (often discounted by utilities) shows which you need. 'Look Like a Scam' compares the price, never accuses a contractor. Safety: keep foam and film away from heat sources and flues.</t>
+          <t>Seven cheap fixes for the drafts that make a house feel cold, set against a typical whole-house insulation quote (blown-in or spray foam often runs several thousand dollars). 1) Door weatherstripping and a door sweep ($10-$25 a door): the biggest felt draft in most homes. 2) Foam gaskets behind outlet and switch covers on outside walls ($5 for a pack). 3) Caulk the window and door trim where it meets the wall ($5-$10 a tube). 4) Window insulation film kits ($15-$25 for several windows) or heavy thermal curtains. 5) Weatherstrip and insulate the attic hatch or pull-down stairs ($20-$50 DIY, $50-$150 for a ready-made stair cover): often a big hole in the ceiling. 6) Seal the basement rim joist with canned foam ($5-$10 a can). 7) Close the fireplace damper or fit a chimney plug ($30-$80) only once the fire and embers are completely out and cold, usually the next day; never on a gas-log fireplace (its damper must stay open); take the plug out before every fire; never block a flue a furnace or water heater vents into. Honest framing: these stop air leaks, which cause most of the 'cold house' feeling; they don't replace insulation in a truly empty wall or attic, and an energy audit (often discounted by utilities) shows which you need. 'Look Like a Scam' compares the price, never accuses a contractor or implies insulation quotes are actual scams. Safety: keep foam and film away from heat sources and flues; with an older natural-draft furnace or water heater, tightening the house can cause CO backdrafting, so get a combustion safety test and keep CO alarms working.</t>
         </is>
       </c>
     </row>
@@ -662,7 +662,7 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>A 1,500-watt space heater draws about 12.5 amps for hours, close to the limit of a standard 15-amp circuit, so the weak point is the connection, not the heater. Never plug it into: 1) an extension cord (most household cords are rated far below that load and heat up, especially coiled or under a rug); 2) a power strip or surge protector (not built for continuous heater loads; most heater manuals say so); 3) a multi-plug adapter or cube tap; 4) a smart plug or timer not rated for the full load (check the rating; many are not); 5) a loose, worn or discolored outlet (a loose plug heats at the contacts and melts). Plug it straight into a wall outlet, ideally on a circuit with nothing else big on it, and check the plug after an hour: warm is normal, hot is not. Also: keep 3 feet clear of anything that can burn, never run it while sleeping or away, and look for tip-over and overheat shutoff and a safety listing (UL, ETL or CSA). Facts to verify at scripting: the NFPA share of home heating fires and deaths involving space heaters (roughly a third of the fires and most of the deaths in recent NFPA reports).</t>
+          <t>A 1,500-watt space heater draws about 12.5 amps for hours, above the 12 amps a 15-amp circuit is meant to carry continuously (the electrical code's 80% rule for continuous loads), so the weak point is the connection, not the heater. Never plug it into: 1) an extension cord (many light-duty household cords, 16- and 18-gauge, are rated only 10-13 amps and heat up, especially coiled or under a rug); 2) a power strip or surge protector (not built for continuous heater loads; most heater manuals say so); 3) a multi-plug adapter or cube tap; 4) a smart plug or timer not rated for the full load (check the rating; many are not); 5) a loose, worn or discolored outlet (a loose plug heats at the contacts and melts). Plug it straight into a wall outlet, ideally on a circuit with nothing else big on it, and check the plug after an hour: warm is normal, hot is not. Also: keep 3 feet clear of anything that can burn, never run it while sleeping or away, and look for tip-over and overheat shutoff and a safety listing (UL, ETL or CSA). Fact for the script: space heaters (fixed and portable) were involved in about one-third of US home heating fires but 88% of home heating fire deaths (NFPA, 2016-2020 annual averages). CPSC, the Red Cross and ESFI all say plug directly into the wall.</t>
         </is>
       </c>
     </row>
@@ -679,7 +679,7 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>The part is the flame sensor: a thin metal rod in the burner flame that proves to the control board the gas lit. When it's coated with carbon or oxide, the board can't read the flame, so the furnace lights, runs a few seconds, shuts the gas off and retries, sometimes locking out after three tries. A new sensor costs about $10-$25; a service call to clean or replace it often runs $150-$300. The fix: turn off power at the furnace switch (and let it cool), remove the burner door, take out the one screw holding the sensor, pull it out by its base, polish the rod lightly with fine emery cloth, fine steel wool or a scouring pad (not coarse sandpaper), wipe it, reinstall, restore power and watch a full cycle. If it still shuts off, other causes: a dirty filter (high limit), a clogged condensate trap or vent pipe (pressure switch), a weak igniter, or a bad sensor wire; that's when to call a tech. Safety: never touch the hot-surface igniter next to it (fragile, skin oils crack it); if you smell gas, stop and call the gas company. Prices as rounded ranges.</t>
+          <t>The part is the flame sensor: a thin metal rod in the burner flame that proves to the control board the gas lit. When it's coated with carbon or oxide, the board can't read the flame, so the furnace lights, runs a few seconds, shuts the gas off and retries, sometimes locking out after three tries. A new sensor costs about $10-$25; a service call to clean or replace it typically runs $100-$250, $300 or more after hours. The fix: turn off power at the furnace switch and turn the gas valve off (and let it cool), remove the burner door, take out the one screw holding the sensor, pull it out by its base, polish the rod lightly with a Scotch-Brite pad or very fine emery cloth (not coarse sandpaper; keep grit off the ceramic), wipe it, reinstall, restore power and watch a full cycle. If it still shuts off, other causes: a dirty filter (high limit), a clogged condensate trap or vent pipe (pressure switch), a weak igniter, or a bad sensor wire; that's when to call a tech. Safety: never touch the hot-surface igniter next to it (fragile, skin oils crack it); if you smell gas, stop and call the gas company. Prices as rounded ranges.</t>
         </is>
       </c>
     </row>
@@ -696,7 +696,7 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Most ceiling fans have a small direction switch on the motor housing (or a reverse button on the remote). In summer the fan should turn counterclockwise looking up, pushing air down for a cooling breeze. In winter, switch it to clockwise on the lowest speed: it pulls air up and pushes the warm air that collects at the ceiling back down the walls without a draft. The U.S. Department of Energy recommends this winter setting. It helps most in rooms with high or vaulted ceilings, where the air near the ceiling can be several degrees warmer than at the floor; in a low-ceiling room the gain is small. The payoff: the room feels warmer at the same thermostat setting, so many people can set it a degree or two lower (the DOE's setback figure works out to roughly 1% a year per degree for 8 hours a day; keep the claim soft, never 'cuts your bill'). How: turn the fan off, wait for it to stop, flip the switch, run it on low. Costs: nothing. Don't run fans in empty rooms; a fan cools people, not rooms. Clean the blades first, since a winter's dust gets thrown around.</t>
+          <t>Most ceiling fans have a small direction switch on the motor housing (or a reverse button on the remote). In summer the fan should turn counterclockwise looking up, pushing air down for a cooling breeze. In winter, switch it to clockwise on the lowest speed: it pulls air up and pushes the warm air that collects at the ceiling back down the walls without a draft. The U.S. Department of Energy recommends this winter setting. It helps most in rooms with high or vaulted ceilings, where the air near the ceiling can be several degrees warmer than at the floor; in a low-ceiling room the gain is small. The payoff: the room feels warmer at the same thermostat setting, so many people can set it a degree or two lower (the DOE's setback figure works out to roughly 1% a year per degree for 8 hours a day; keep the claim soft, never 'cuts your bill'). How: turn the fan off, wait for it to stop, flip the switch, run it on low. Costs: nothing. Turn it off when nobody's in the room. The brief follows DOE and ENERGY STAR guidance; check the reference video's own view of reverse mode before quoting it. Clean the blades first, since a winter's dust gets thrown around.</t>
         </is>
       </c>
     </row>
@@ -713,7 +713,7 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>In a winter outage, a gas furnace won't run without power for its blower, inducer and igniter, but it only needs about 300-800 watts. A car's battery and alternator can supply that through a pure sine wave inverter (about $100-$250 for a 1,000-1,500 watt model) clamped to the battery, with the engine running to keep it charged; a hybrid can run for many hours on little fuel (an idling car typically burns roughly a quarter to half a gallon an hour). The furnace has to be connectable: most are hard-wired, so an electrician installs a furnace power inlet or transfer switch (often $150-$400) that lets you plug it in safely; never backfeed a house panel or wire around a switch. Safety above all: the car runs outside in open air, never in a garage, even with the door open, because of carbon monoxide; run the cord through a window cracked open, with a CO detector inside on every floor; use an outdoor-rated cord of the right gauge. Honest limits: it runs the furnace, not the whole house; a modified-sine inverter can damage some furnace boards. Compare: a portable generator runs $500-$1,500 plus fuel and storage, a standby generator $7,000-$15,000+ installed.</t>
+          <t>In a winter outage, a gas furnace won't run without power for its blower, inducer and igniter, but it only needs about 300-800 watts. A car's battery and alternator can supply that through a pure sine wave inverter (about $100-$250 for a 1,000-1,500 watt model) clamped to the battery, with the engine running to keep it charged; a hybrid can run for many hours on little fuel (an idling car typically burns roughly a quarter to half a gallon an hour). The furnace has to be connectable: most are hard-wired, so an electrician installs a furnace power inlet or single-circuit transfer switch (often $200-$500) that lets you plug it in safely; never backfeed a house panel or wire around a switch. Safety above all: the car runs outside in open air, never in a garage, even with the door open, because of carbon monoxide; park with the tailpipe pointing away from the house, at least 20 feet from doors, windows and vents (CPSC's distance for generators), keep the tailpipe clear of snow, never sit or sleep in the idling car; bring the cord in without leaving a gap (close the window or door on it and seal the gap, or use the inlet the electrician fits); CO alarms on every level; an outdoor-rated cord of the right gauge. Honest limits: it runs the furnace, not the whole house; a modified-sine inverter can damage some furnace boards, and some furnaces won't light on an inverter whose neutral isn't bonded to ground (the flame sensor needs that reference, and polarity must be right): the electrician fitting the inlet can sort it out. Compare: a portable generator runs $500-$1,500 plus fuel and storage, a standby generator $7,000-$15,000+ installed.</t>
         </is>
       </c>
     </row>

</xml_diff>